<commit_message>
Update Feefo and Review reports for 2026-01-19T01:47:54Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1003991</t>
+          <t>1062346</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,71 +480,71 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1003991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1039106</t>
+          <t>1084121</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1039106&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1062124</t>
+          <t>1088335</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062124&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088335&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1084121</t>
+          <t>1088991</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1100632</t>
+          <t>1093803</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,52 +556,52 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1100632&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1116877</t>
+          <t>1098821</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1116877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1098821&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1149454</t>
+          <t>1120730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1149454&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1120730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1152259</t>
+          <t>1141180</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,52 +613,52 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1141180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1209526</t>
+          <t>1150628</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1211012</t>
+          <t>1169338</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1211012&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1169338&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1177804</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1177804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1238199</t>
+          <t>1179336</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1238199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179336&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1254182</t>
+          <t>1213412</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1254182&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1261485</t>
+          <t>1232243</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1261485&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1276718</t>
+          <t>1234030</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1276718&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234030&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1312519</t>
+          <t>1240077</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,52 +765,52 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312519&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1240077&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1345877</t>
+          <t>1240712</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1240712&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1353406</t>
+          <t>1246450</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1353406&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1246450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1359908</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359908&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1383055</t>
+          <t>1251013</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1383055&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1251013&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1404078</t>
+          <t>1262539</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404078&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1262539&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1418337</t>
+          <t>1268629</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1418337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1268629&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1281427</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1281427&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1458881</t>
+          <t>1307555</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,33 +917,33 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1458881&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1491886</t>
+          <t>1311523</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311523&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1505198</t>
+          <t>1321536</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,71 +955,71 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1321536&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1508457</t>
+          <t>1345877</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508457&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1513080</t>
+          <t>1347117</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1513080&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1526808</t>
+          <t>1354859</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526808&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1534682</t>
+          <t>1359921</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1534682&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359921&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1545611</t>
+          <t>1384307</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,14 +1050,14 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1545611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1384307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1570250</t>
+          <t>1401261</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,52 +1069,52 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1401261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>350209</t>
+          <t>1421476</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=350209&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1421476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>352545</t>
+          <t>1423470</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1423470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>427505</t>
+          <t>1430188</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,33 +1126,33 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=427505&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430188&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>431082</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=431082&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>463104</t>
+          <t>1439606</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1164,33 +1164,33 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=463104&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1439606&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1453636</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1453636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>1454208</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1202,14 +1202,14 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1454208&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>638637</t>
+          <t>1470930</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,14 +1221,14 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=638637&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1470930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>730583</t>
+          <t>1480636</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1240,14 +1240,14 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1480636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>755080</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1259,14 +1259,14 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=755080&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>824644</t>
+          <t>1491886</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,52 +1278,52 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>848767</t>
+          <t>1492721</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848767&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1492721&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>882806</t>
+          <t>1500484</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882806&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>905169</t>
+          <t>1502594</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,33 +1335,33 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>937471</t>
+          <t>1505198</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>945255</t>
+          <t>1507470</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,33 +1373,33 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>960885</t>
+          <t>1508457</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=960885&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508457&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>963663</t>
+          <t>1537066</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -1411,7 +1411,672 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963663&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537066&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1543312</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1547383</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547383&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1561674</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>159976</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>352545</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>418373</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=418373&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>458823</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>2</v>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=458823&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="n">
+        <v>5</v>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>486442</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=486442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>498516</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=498516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>499724</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>3</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>501968</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=501968&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>527736</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=527736&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="n">
+        <v>3</v>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>571200</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>3</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>578486</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>621809</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>6</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>630609</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=630609&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>729389</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=729389&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>730583</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>744558</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=744558&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>768387</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768387&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>786481</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>4</v>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>788669</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=788669&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>848232</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>860698</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>880642</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>904462</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=904462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>905169</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>911076</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=911076&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>932785</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=932785&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>963254</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963254&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>967090</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=967090&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>991741</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-01-26T01:49:54Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1062346</t>
+          <t>1025557</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,33 +480,33 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1025557&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1084121</t>
+          <t>1029754</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029754&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1088335</t>
+          <t>1039106</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088335&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1039106&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1088991</t>
+          <t>1056980</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1056980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1093803</t>
+          <t>1152259</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1098821</t>
+          <t>1162292</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1098821&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1120730</t>
+          <t>1174183</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1120730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1174183&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1141180</t>
+          <t>1176044</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,52 +613,52 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1141180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1150628</t>
+          <t>1179458</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1169338</t>
+          <t>1184330</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1169338&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1177804</t>
+          <t>1193213</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1177804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1193213&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1179336</t>
+          <t>1225269</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179336&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1225269&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1213412</t>
+          <t>1232243</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1244126</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244126&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1234030</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234030&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1240077</t>
+          <t>1264171</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1240077&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1264171&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1240712</t>
+          <t>1267884</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,33 +784,33 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1240712&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1267884&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1246450</t>
+          <t>1277156</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1246450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1277156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1292768</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1292768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1251013</t>
+          <t>1309371</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1251013&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1309371&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1262539</t>
+          <t>1328533</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1262539&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1328533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1268629</t>
+          <t>1334910</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1268629&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1281427</t>
+          <t>1345002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1281427&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345002&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1307555</t>
+          <t>1345877</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1311523</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311523&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1321536</t>
+          <t>1352064</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,33 +955,33 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1321536&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1352064&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1345877</t>
+          <t>1361978</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1347117</t>
+          <t>1365791</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,33 +993,33 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1354859</t>
+          <t>1372828</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1359921</t>
+          <t>1395590</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,33 +1031,33 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359921&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1395590&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1384307</t>
+          <t>1418337</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1384307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1418337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1401261</t>
+          <t>1424795</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1401261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1424795&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1421476</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1421476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1423470</t>
+          <t>1432966</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1423470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1432966&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1430188</t>
+          <t>1438876</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,33 +1126,33 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430188&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1438876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1455504</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1455504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1439606</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1164,52 +1164,52 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1439606&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1453636</t>
+          <t>1498910</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1453636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1454208</t>
+          <t>1508457</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1454208&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508457&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1470930</t>
+          <t>1525839</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,33 +1221,33 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1470930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525839&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1480636</t>
+          <t>1537066</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1480636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537066&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1540005</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1259,14 +1259,14 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1540005&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1491886</t>
+          <t>1543312</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,52 +1278,52 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1492721</t>
+          <t>1547810</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1492721&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547810&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1500484</t>
+          <t>1555205</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1555205&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1502594</t>
+          <t>1560354</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560354&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1505198</t>
+          <t>1573029</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,14 +1354,14 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1573029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1507470</t>
+          <t>159976</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,14 +1373,14 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1508457</t>
+          <t>298443</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1392,52 +1392,52 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508457&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=298443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1537066</t>
+          <t>350209</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537066&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=350209&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1543312</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1547383</t>
+          <t>484197</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -1449,14 +1449,14 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547383&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=484197&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1561674</t>
+          <t>510518</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1468,33 +1468,33 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510518&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>159976</t>
+          <t>582818</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=582818&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>352545</t>
+          <t>616288</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -1506,33 +1506,33 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=616288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>418373</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=418373&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>458823</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -1544,33 +1544,33 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=458823&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>821096</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=821096&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>486442</t>
+          <t>830584</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -1582,14 +1582,14 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=486442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>498516</t>
+          <t>845468</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1601,52 +1601,52 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=498516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=845468&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>857942</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>501968</t>
+          <t>869313</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=501968&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=869313&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>527736</t>
+          <t>876141</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -1658,52 +1658,52 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=527736&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>881907</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>571200</t>
+          <t>905169</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>578486</t>
+          <t>986868</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -1715,368 +1715,26 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=986868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>999592</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>630609</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="n">
-        <v>2</v>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=630609&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>729389</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="n">
-        <v>2</v>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=729389&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>730583</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="n">
-        <v>2</v>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>744558</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="n">
-        <v>2</v>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=744558&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>768387</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="n">
-        <v>2</v>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768387&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>786481</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="n">
-        <v>4</v>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>788669</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=788669&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>848232</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="n">
-        <v>2</v>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>860698</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="n">
-        <v>2</v>
-      </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>876141</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="n">
-        <v>2</v>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>880642</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="n">
-        <v>2</v>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>904462</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="n">
-        <v>2</v>
-      </c>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=904462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>905169</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="n">
-        <v>3</v>
-      </c>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>911076</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="n">
-        <v>2</v>
-      </c>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=911076&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>932785</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="n">
-        <v>2</v>
-      </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=932785&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>963254</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="n">
-        <v>2</v>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963254&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>967090</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="n">
-        <v>2</v>
-      </c>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=967090&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>991741</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="n">
-        <v>2</v>
-      </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-02-02T02:03:27Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1025557</t>
+          <t>1049381</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,90 +480,90 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1025557&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1029754</t>
+          <t>1062175</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029754&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062175&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1039106</t>
+          <t>1088991</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1039106&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1056980</t>
+          <t>1093803</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1056980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1152259</t>
+          <t>1116877</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1116877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1162292</t>
+          <t>1150628</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1174183</t>
+          <t>1162292</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,7 +594,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1174183&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
@@ -620,7 +620,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1179458</t>
+          <t>1184330</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1184330</t>
+          <t>1184431</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1193213</t>
+          <t>1213412</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1193213&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1225269</t>
+          <t>1228498</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1225269&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1228498&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1231622</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,52 +708,52 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1231622&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1244126</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244126&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1261865</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1261865&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1264171</t>
+          <t>1299895</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1264171&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1299895&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1267884</t>
+          <t>1322572</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1267884&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1277156</t>
+          <t>1323524</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1277156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1323524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1292768</t>
+          <t>1340963</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1292768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1340963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1309371</t>
+          <t>1356778</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1309371&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1328533</t>
+          <t>1365791</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1328533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1334910</t>
+          <t>1375255</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1345002</t>
+          <t>1378864</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345002&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1378864&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1345877</t>
+          <t>1388105</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1388105&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1418337</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1418337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1352064</t>
+          <t>1420726</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,14 +955,14 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1352064&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1420726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1361978</t>
+          <t>1425892</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,14 +974,14 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1425892&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1365791</t>
+          <t>1429965</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,33 +993,33 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1429965&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1372828</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1395590</t>
+          <t>1433516</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1395590&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1433516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1418337</t>
+          <t>1435597</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,14 +1050,14 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1418337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1424795</t>
+          <t>1466386</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1424795&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466386&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1477967</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477967&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1432966</t>
+          <t>1481251</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1432966&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1481251&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1438876</t>
+          <t>1483521</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,52 +1126,52 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1438876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1455504</t>
+          <t>1486879</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1455504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486879&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1491886</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1498910</t>
+          <t>1500484</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,33 +1183,33 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1508457</t>
+          <t>1508805</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508457&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1525839</t>
+          <t>1519522</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,33 +1221,33 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525839&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1519522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1537066</t>
+          <t>1526808</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537066&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526808&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1540005</t>
+          <t>1534682</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1259,52 +1259,52 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1540005&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1534682&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1543312</t>
+          <t>1541888</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541888&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1547810</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547810&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1555205</t>
+          <t>1560710</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -1316,14 +1316,14 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1555205&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1560354</t>
+          <t>1562842</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560354&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1573029</t>
+          <t>1566071</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,14 +1354,14 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1573029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1566071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>159976</t>
+          <t>258379</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,14 +1373,14 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=258379&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>298443</t>
+          <t>460660</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1392,71 +1392,71 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=298443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>350209</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=350209&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>482198</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=482198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>484197</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=484197&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>510518</t>
+          <t>554644</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510518&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=554644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>616288</t>
+          <t>611125</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=616288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=611125&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>701046</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -1544,14 +1544,14 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=701046&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>821096</t>
+          <t>767926</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -1563,33 +1563,33 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=821096&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>830584</t>
+          <t>768730</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>845468</t>
+          <t>811253</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1601,14 +1601,14 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=845468&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=811253&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>857942</t>
+          <t>824644</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -1620,33 +1620,33 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>869313</t>
+          <t>848232</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=869313&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>856677</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -1658,14 +1658,14 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=856677&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>881907</t>
+          <t>857942</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -1677,52 +1677,52 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>905169</t>
+          <t>875307</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=875307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>986868</t>
+          <t>876141</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=986868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>999592</t>
+          <t>905169</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -1734,6 +1734,139 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>908011</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908011&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>915286</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>917255</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=917255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>930044</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>945255</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>949916</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=949916&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
           <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-02-09T02:04:46Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1049381</t>
+          <t>100458</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,71 +480,71 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1062175</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062175&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1088991</t>
+          <t>1062346</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1093803</t>
+          <t>1078657</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1078657&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1116877</t>
+          <t>1093185</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1116877&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1150628</t>
+          <t>1093508</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093508&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1162292</t>
+          <t>1107283</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1176044</t>
+          <t>1135028</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135028&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1184330</t>
+          <t>1156573</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1156573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1184431</t>
+          <t>1169338</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1169338&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1213412</t>
+          <t>1176044</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1228498</t>
+          <t>1180755</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1228498&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1180755&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1231622</t>
+          <t>1181236</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,33 +708,33 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1231622&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1183385</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183385&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1261865</t>
+          <t>1184205</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1261865&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184205&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1299895</t>
+          <t>1184330</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1299895&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1322572</t>
+          <t>1198294</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1323524</t>
+          <t>1245610</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1323524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1245610&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1340963</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1340963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1356778</t>
+          <t>1278602</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1365791</t>
+          <t>1284696</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1284696&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1375255</t>
+          <t>1300288</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1300288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1378864</t>
+          <t>1311530</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1378864&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311530&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1388105</t>
+          <t>1329593</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,71 +917,71 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1388105&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329593&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1418337</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1418337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1420726</t>
+          <t>1353406</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1420726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1353406&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1425892</t>
+          <t>1356778</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1425892&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1429965</t>
+          <t>1372828</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,33 +993,33 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1429965&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1375803</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1433516</t>
+          <t>1399796</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,33 +1031,33 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1433516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1399796&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1435597</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1466386</t>
+          <t>1455504</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466386&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1455504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1477967</t>
+          <t>1465349</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477967&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1465349&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1481251</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1481251&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1483521</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,45 +1126,45 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1486879</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486879&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1491886</t>
+          <t>1494582</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494582&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
@@ -1209,7 +1209,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1519522</t>
+          <t>1525839</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,7 +1221,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1519522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525839&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
@@ -1247,26 +1247,26 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1534682</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1534682&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1541888</t>
+          <t>1549666</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,33 +1278,33 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541888&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1549666&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1561674</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1560710</t>
+          <t>1570250</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -1316,14 +1316,14 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1562842</t>
+          <t>1570445</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570445&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1566071</t>
+          <t>224266</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,14 +1354,14 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1566071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=224266&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>258379</t>
+          <t>264469</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,14 +1373,14 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=258379&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=264469&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>460660</t>
+          <t>355476</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1392,83 +1392,83 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=355476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>476768</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=476768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>482198</t>
+          <t>479583</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=482198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=479583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>489068</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=489068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>554644</t>
+          <t>578486</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=554644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -1494,64 +1494,64 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>611125</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=611125&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>730583</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>701046</t>
+          <t>768730</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=701046&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>767926</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -1563,33 +1563,33 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>768730</t>
+          <t>831596</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=831596&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>811253</t>
+          <t>832462</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1601,14 +1601,14 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=811253&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=832462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>824644</t>
+          <t>833691</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -1620,14 +1620,14 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=833691&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>848232</t>
+          <t>866983</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -1639,52 +1639,52 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=866983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>856677</t>
+          <t>885034</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=856677&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=885034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>857942</t>
+          <t>905169</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>875307</t>
+          <t>945255</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -1696,14 +1696,14 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=875307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>957539</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -1715,159 +1715,7 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>905169</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="n">
-        <v>4</v>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>908011</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="n">
-        <v>2</v>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908011&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="n">
-        <v>4</v>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>917255</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="n">
-        <v>2</v>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=917255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>930044</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="n">
-        <v>2</v>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>945255</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="n">
-        <v>3</v>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>949916</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="n">
-        <v>2</v>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=949916&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=957539&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-02-16T02:05:02Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,7 +475,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
@@ -487,7 +487,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1009086</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,52 +499,52 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1062346</t>
+          <t>1012276</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1012276&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1078657</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1078657&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1093185</t>
+          <t>1029103</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029103&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1093508</t>
+          <t>1047587</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093508&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1107283</t>
+          <t>1088991</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1135028</t>
+          <t>1107283</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135028&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1156573</t>
+          <t>1135028</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1156573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135028&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1169338</t>
+          <t>1135146</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1169338&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135146&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1176044</t>
+          <t>1159199</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1159199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1180755</t>
+          <t>1160907</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1180755&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1181236</t>
+          <t>1179458</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1183385</t>
+          <t>1185231</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183385&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1185231&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1184205</t>
+          <t>1234030</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,52 +746,52 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184205&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234030&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1184330</t>
+          <t>1234780</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184330&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234780&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1198294</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1245610</t>
+          <t>1279006</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1245610&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1279006&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1290730</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1278602</t>
+          <t>1290822</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290822&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1284696</t>
+          <t>1292773</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1284696&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1292773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1300288</t>
+          <t>1298088</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1300288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1298088&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1311530</t>
+          <t>1302008</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311530&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1302008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1329593</t>
+          <t>1311546</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329593&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311546&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1322572</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,71 +936,71 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1353406</t>
+          <t>1340309</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1353406&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1340309&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1356778</t>
+          <t>1341118</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341118&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1372828</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1375803</t>
+          <t>1351353</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351353&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1399796</t>
+          <t>1354859</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,71 +1031,71 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1399796&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1356288</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1455504</t>
+          <t>1356778</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1455504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1465349</t>
+          <t>1357491</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1465349&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1357491&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1466482</t>
+          <t>1360194</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360194&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1365342</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,52 +1126,52 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1365791</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1494582</t>
+          <t>1369499</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494582&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1369499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1500484</t>
+          <t>1372929</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,33 +1183,33 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1508805</t>
+          <t>1376957</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1376957&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1525839</t>
+          <t>1401261</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,52 +1221,52 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525839&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1401261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1526808</t>
+          <t>1466430</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526808&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466430&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1466437</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466437&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1549666</t>
+          <t>1466442</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,14 +1278,14 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1549666&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1561674</t>
+          <t>1466708</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -1297,33 +1297,33 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466708&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1570250</t>
+          <t>1474234</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1474234&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1570445</t>
+          <t>1475320</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570445&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1475320&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>224266</t>
+          <t>1477424</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,14 +1354,14 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=224266&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477424&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>264469</t>
+          <t>1478443</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,14 +1373,14 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=264469&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>355476</t>
+          <t>1483518</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1392,33 +1392,33 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=355476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483518&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>476768</t>
+          <t>1483521</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=476768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>479583</t>
+          <t>1487795</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -1430,52 +1430,52 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=479583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487795&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>489068</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=489068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>578486</t>
+          <t>1497676</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>582818</t>
+          <t>1502113</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -1487,33 +1487,33 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=582818&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>1507470</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>730583</t>
+          <t>1536454</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -1525,52 +1525,52 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536454&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>768730</t>
+          <t>1537657</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537657&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>1539715</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>831596</t>
+          <t>1539740</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -1582,14 +1582,14 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=831596&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539740&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>832462</t>
+          <t>1543063</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1601,14 +1601,14 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=832462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543063&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>833691</t>
+          <t>1543312</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -1620,71 +1620,71 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=833691&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>866983</t>
+          <t>1553515</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=866983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553515&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>885034</t>
+          <t>1562842</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=885034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>905169</t>
+          <t>1572868</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1572868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>945255</t>
+          <t>1574098</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -1696,26 +1696,691 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574098&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>957539</t>
+          <t>1574947</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=957539&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574947&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1575476</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>4</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1575956</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575956&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1576267</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576267&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1576271</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576271&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1580749</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580749&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>348289</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=348289&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>360873</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=360873&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>463104</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=463104&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>476768</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=476768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>512339</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=512339&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>530476</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=530476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>551379</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=551379&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>578486</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>621809</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="n">
+        <v>3</v>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>665054</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="n">
+        <v>3</v>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=665054&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>688997</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=688997&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>713987</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=713987&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>734624</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=734624&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>759749</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=759749&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>767562</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767562&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>767926</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>830584</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>839295</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=839295&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>846598</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=846598&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>865097</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>905169</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="n">
+        <v>4</v>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>910678</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=910678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>917255</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=917255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>920040</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>929844</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=929844&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>944163</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944163&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>982044</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=982044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>998926</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="n">
+        <v>3</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=998926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-02-23T02:04:59Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,45 +468,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100458</t>
+          <t>1006389</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1006389&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1009086</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1012276</t>
+          <t>1073876</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,33 +518,33 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1012276&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1073876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1084121</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1029103</t>
+          <t>1093185</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029103&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1047587</t>
+          <t>1129242</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1129242&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1088991</t>
+          <t>1134991</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1134991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1107283</t>
+          <t>1135028</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135028&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1135028</t>
+          <t>1135146</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135028&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135146&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1135146</t>
+          <t>1178765</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1135146&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1178765&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1159199</t>
+          <t>1225149</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1159199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1225149&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1160907</t>
+          <t>1232243</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1179458</t>
+          <t>1265734</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1265734&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1185231</t>
+          <t>1290730</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1185231&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1234030</t>
+          <t>1298088</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,223 +746,223 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234030&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1298088&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1234780</t>
+          <t>1305084</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234780&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1305084&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1322617</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322617&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1279006</t>
+          <t>1356288</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1279006&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1290730</t>
+          <t>1356778</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1290822</t>
+          <t>1357491</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290822&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1357491&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1292773</t>
+          <t>1359179</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1292773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359179&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1298088</t>
+          <t>1360194</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1298088&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360194&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1302008</t>
+          <t>1360290</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1302008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360290&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1311546</t>
+          <t>1361711</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1311546&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361711&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1322572</t>
+          <t>1365122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1340309</t>
+          <t>1365791</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1340309&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1341118</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,33 +974,33 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341118&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1395590</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1395590&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1351353</t>
+          <t>1414677</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351353&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1414677&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1354859</t>
+          <t>1423447</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,147 +1031,147 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1423447&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1356288</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356288&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1356778</t>
+          <t>1457936</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1457936&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1357491</t>
+          <t>1459180</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1357491&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1459180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1360194</t>
+          <t>1466430</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360194&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466430&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1365342</t>
+          <t>1466437</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466437&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1365791</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1369499</t>
+          <t>1466708</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1369499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466708&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1372929</t>
+          <t>1470650</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,90 +1183,90 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1470650&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1376957</t>
+          <t>1474234</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1376957&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1474234&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1401261</t>
+          <t>1476097</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1401261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1466430</t>
+          <t>1477424</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466430&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477424&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1466437</t>
+          <t>1477967</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466437&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477967&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1466442</t>
+          <t>1483520</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,14 +1278,14 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483520&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1466708</t>
+          <t>1485956</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -1297,33 +1297,33 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466708&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485956&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1474234</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1474234&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1475320</t>
+          <t>1500484</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1475320&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1477424</t>
+          <t>1502113</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,14 +1354,14 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477424&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1478443</t>
+          <t>1509775</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1373,14 +1373,14 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1509775&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1483518</t>
+          <t>1510344</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1392,33 +1392,33 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483518&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1510344&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1483521</t>
+          <t>1512876</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1512876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1487795</t>
+          <t>1513071</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -1430,33 +1430,33 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487795&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1513071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1548271</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1548271&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1497676</t>
+          <t>1561674</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1468,14 +1468,14 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1502113</t>
+          <t>156570</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -1487,33 +1487,33 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=156570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1507470</t>
+          <t>1572868</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1572868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1536454</t>
+          <t>1574692</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -1525,52 +1525,52 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536454&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1537657</t>
+          <t>1575950</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1537657&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575950&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1539715</t>
+          <t>1575956</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575956&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1539740</t>
+          <t>1577935</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -1582,109 +1582,109 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539740&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1577935&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1543063</t>
+          <t>1580749</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543063&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580749&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1543312</t>
+          <t>1582651</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1582651&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1553515</t>
+          <t>213148</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553515&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=213148&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1562842</t>
+          <t>352545</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1572868</t>
+          <t>460660</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1572868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1574098</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -1696,71 +1696,71 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574098&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1574947</t>
+          <t>478341</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574947&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=478341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1575476</t>
+          <t>551379</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=551379&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1575956</t>
+          <t>577930</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575956&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=577930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1576267</t>
+          <t>597698</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -1772,14 +1772,14 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576267&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=597698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1576271</t>
+          <t>665054</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
@@ -1791,52 +1791,52 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576271&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=665054&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1580749</t>
+          <t>679514</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580749&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=679514&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>348289</t>
+          <t>698774</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=348289&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=698774&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>360873</t>
+          <t>706455</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
@@ -1848,71 +1848,71 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=360873&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=706455&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>463104</t>
+          <t>708521</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=463104&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=708521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>730583</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>476768</t>
+          <t>767926</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=476768&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>512339</t>
+          <t>786483</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -1924,14 +1924,14 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=512339&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>530476</t>
+          <t>787804</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
@@ -1943,33 +1943,33 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=530476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=787804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>551379</t>
+          <t>833691</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=551379&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=833691&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>578486</t>
+          <t>846598</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
@@ -1981,71 +1981,71 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=846598&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>848232</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>665054</t>
+          <t>851722</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=665054&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=851722&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>688997</t>
+          <t>865097</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=688997&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>713987</t>
+          <t>898792</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -2057,14 +2057,14 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=713987&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=898792&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>734624</t>
+          <t>905169</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -2076,14 +2076,14 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=734624&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>759749</t>
+          <t>937471</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -2095,14 +2095,14 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=759749&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>767562</t>
+          <t>974715</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -2114,14 +2114,14 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767562&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=974715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>767926</t>
+          <t>991747</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -2133,14 +2133,14 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=767926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>830584</t>
+          <t>998926</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -2152,14 +2152,14 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=998926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>839295</t>
+          <t>999592</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -2171,216 +2171,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=839295&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>846598</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="n">
-        <v>3</v>
-      </c>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=846598&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>865097</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="n">
-        <v>2</v>
-      </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>905169</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="n">
-        <v>4</v>
-      </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>910678</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="n">
-        <v>2</v>
-      </c>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=910678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>917255</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="n">
-        <v>3</v>
-      </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=917255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>920040</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="n">
-        <v>2</v>
-      </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>929844</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="n">
-        <v>2</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=929844&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>937471</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="n">
-        <v>2</v>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>944163</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="n">
-        <v>2</v>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944163&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>982044</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="n">
-        <v>2</v>
-      </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=982044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>998926</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="n">
-        <v>3</v>
-      </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=998926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-03-09T01:59:43Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1008277</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1008277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1033155</t>
+          <t>1087476</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,52 +499,52 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1033155&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1087476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1087476</t>
+          <t>1093185</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1087476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1107283</t>
+          <t>1102757</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1102757&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1121850</t>
+          <t>1179458</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1121850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1187498</t>
+          <t>1183789</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,52 +575,52 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1187498&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1198294</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1244126</t>
+          <t>1205131</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244126&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1205131&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1249251</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249251&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1296744</t>
+          <t>1301141</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,33 +651,33 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1296744&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1301141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1344943</t>
+          <t>1320773</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1320773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1364739</t>
+          <t>1321783</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1364739&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1321783&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1365791</t>
+          <t>1322572</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1375255</t>
+          <t>1347117</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,71 +727,71 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1408746</t>
+          <t>1353406</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1408746&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1353406&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1356778</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1435597</t>
+          <t>1360293</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360293&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1474811</t>
+          <t>1380407</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,71 +803,71 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1474811&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1380407&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1394198</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1529093</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1550368</t>
+          <t>1445750</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1550368&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1445750&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1551628</t>
+          <t>1459006</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,52 +898,52 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1551628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1459006&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1561674</t>
+          <t>1478506</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1561674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478506&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1575671</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575671&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>238431</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,14 +955,14 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=238431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>460660</t>
+          <t>1509775</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,33 +974,33 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1509775&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>478341</t>
+          <t>236959</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=478341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=236959&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>238431</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=238431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>326441</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,14 +1050,14 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=326441&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>905169</t>
+          <t>352545</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=905169&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>913184</t>
+          <t>460660</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=913184&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>915286</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,33 +1107,33 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>941107</t>
+          <t>499724</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=941107&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>986868</t>
+          <t>510573</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1145,7 +1145,216 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=986868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>826183</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826183&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>844846</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=844846&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>895147</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>901984</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=901984&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>930162</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930162&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>945255</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>974423</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=974423&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>980862</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=980862&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-03-16T02:12:57Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,64 +468,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1008277</t>
+          <t>1005045</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1008277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1005045&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1087476</t>
+          <t>1009086</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1087476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1093185</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1102757</t>
+          <t>1147913</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1102757&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1147913&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1179458</t>
+          <t>1150371</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150371&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1183789</t>
+          <t>1181236</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,45 +575,45 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1198294</t>
+          <t>1183789</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1205131</t>
+          <t>1218093</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1205131&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1218093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
@@ -639,45 +639,45 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1301141</t>
+          <t>1260970</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1301141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1260970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1320773</t>
+          <t>1268384</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1320773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1268384&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1321783</t>
+          <t>1341118</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1321783&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341118&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1322572</t>
+          <t>1344943</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1347117</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1353406</t>
+          <t>1351207</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1353406&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1356778</t>
+          <t>1356252</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356778&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356252&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1360293</t>
+          <t>1367998</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,90 +784,90 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1360293&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1380407</t>
+          <t>1371524</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1380407&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1371524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1373926</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1373926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1394198</t>
+          <t>1374002</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394198&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1374002&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1403944</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1403944&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1445750</t>
+          <t>1404697</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1445750&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404697&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1459006</t>
+          <t>1476097</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,7 +898,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1459006&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1485887</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485887&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1485890</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,14 +955,14 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485890&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1509775</t>
+          <t>1500484</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,52 +974,52 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1509775&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1504952</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1504952&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>236959</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=236959&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>238431</t>
+          <t>1550963</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,33 +1031,33 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=238431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1550963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>326441</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=326441&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>352545</t>
+          <t>498516</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,33 +1069,33 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=498516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>460660</t>
+          <t>499724</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>521049</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,33 +1107,33 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=521049&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>510573</t>
+          <t>569413</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1145,33 +1145,33 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=569413&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>571200</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>826183</t>
+          <t>578486</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,14 +1183,14 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826183&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>844846</t>
+          <t>708521</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1202,33 +1202,33 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=844846&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=708521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>722984</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722984&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>895147</t>
+          <t>722986</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1240,33 +1240,33 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722986&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>901984</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=901984&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>930162</t>
+          <t>826992</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,14 +1278,14 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930162&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826992&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>937471</t>
+          <t>830584</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -1297,33 +1297,33 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>945255</t>
+          <t>852646</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=945255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=852646&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>974423</t>
+          <t>866983</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,26 +1335,273 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=974423&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=866983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>980862</t>
+          <t>876141</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=980862&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>880642</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>881907</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>895147</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>898792</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=898792&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>903313</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=903313&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>915286</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>932785</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=932785&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>943955</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=943955&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>950942</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>2</v>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=950942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>977167</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=977167&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>982044</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=982044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-03-23T02:09:44Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,45 +468,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1005045</t>
+          <t>1001638</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1005045&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1001638&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1009086</t>
+          <t>1007604</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1007604&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1008277</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1008277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1147913</t>
+          <t>1013803</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1147913&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1013803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1150371</t>
+          <t>1015762</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150371&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1015762&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1181236</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1183789</t>
+          <t>1076391</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,71 +594,71 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1076391&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1218093</t>
+          <t>1088991</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1218093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1093508</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093508&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1260970</t>
+          <t>1121850</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1260970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1121850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1268384</t>
+          <t>1130272</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,71 +670,71 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1268384&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1130272&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1341118</t>
+          <t>1136421</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341118&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1136421&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1344943</t>
+          <t>1148799</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1148799&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1150371</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150371&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1351207</t>
+          <t>1154087</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1154087&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1356252</t>
+          <t>1158524</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,71 +765,71 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1356252&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1158524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1367998</t>
+          <t>1172375</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1172375&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1371524</t>
+          <t>1174703</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1371524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1174703&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1373926</t>
+          <t>1183789</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1373926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1183789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1374002</t>
+          <t>1205131</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1374002&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1205131&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1403944</t>
+          <t>1260970</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1403944&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1260970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1404697</t>
+          <t>1281427</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404697&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1281427&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1476097</t>
+          <t>1320773</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1320773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1478506</t>
+          <t>1327665</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,71 +917,71 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478506&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1327665&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1485887</t>
+          <t>1328533</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485887&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1328533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1485890</t>
+          <t>1344943</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485890&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1500484</t>
+          <t>1355692</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1355692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1504952</t>
+          <t>1365394</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,33 +993,33 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1504952&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1365394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1367998</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1550963</t>
+          <t>1369763</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,33 +1031,33 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1550963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1369763&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1373777</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1373777&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>498516</t>
+          <t>1373926</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=498516&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1373926&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>1374002</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1374002&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>521049</t>
+          <t>1397797</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=521049&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1397797&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>1397881</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,33 +1126,33 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1397881&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>569413</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=569413&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>571200</t>
+          <t>1438101</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1164,14 +1164,14 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1438101&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>578486</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,14 +1183,14 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=578486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>708521</t>
+          <t>1477487</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1202,33 +1202,33 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=708521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1477487&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>722984</t>
+          <t>1478303</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722984&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478303&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>722986</t>
+          <t>1478663</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1240,14 +1240,14 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722986&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478663&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>1482056</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1259,14 +1259,14 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1482056&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>826992</t>
+          <t>1482683</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1278,52 +1278,52 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826992&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1482683&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>830584</t>
+          <t>1485887</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485887&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>852646</t>
+          <t>1486524</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=852646&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>866983</t>
+          <t>1486947</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1335,14 +1335,14 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=866983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486947&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>1488678</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1354,90 +1354,90 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>880642</t>
+          <t>1490131</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490131&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>881907</t>
+          <t>1490570</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>895147</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>898792</t>
+          <t>1490590</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=898792&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490590&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>903313</t>
+          <t>1497862</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -1449,14 +1449,14 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=903313&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497862&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>915286</t>
+          <t>1500484</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1468,14 +1468,14 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500484&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>932785</t>
+          <t>1500493</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -1487,33 +1487,33 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=932785&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500493&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>937471</t>
+          <t>1507470</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>943955</t>
+          <t>1524113</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -1525,14 +1525,14 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=943955&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1524113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>950942</t>
+          <t>1539740</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -1544,62 +1544,860 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=950942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539740&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>977167</t>
+          <t>1543312</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=977167&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1543312&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>982044</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=982044&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>999592</t>
+          <t>1550056</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1550056&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1554394</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1554394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1557703</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1557703&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1560710</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1567751</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="n">
+        <v>3</v>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567751&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1567787</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567787&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1582443</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1582443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>168041</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>2</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=168041&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>260606</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=260606&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>355476</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=355476&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>358464</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=358464&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>442549</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=442549&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>455575</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=455575&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>10</v>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>493192</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=493192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>499724</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>504064</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=504064&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>528850</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=528850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>629528</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=629528&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>689351</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=689351&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>752563</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752563&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>768387</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768387&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>786481</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>4</v>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>819982</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=819982&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>824644</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>848232</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>850377</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=850377&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>860698</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>879362</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879362&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>895147</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>5</v>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>896464</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=896464&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>903313</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="n">
+        <v>5</v>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=903313&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>915286</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>925318</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=925318&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>929871</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="n">
+        <v>3</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=929871&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>944805</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>957539</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="n">
+        <v>3</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=957539&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>971116</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="n">
+        <v>3</v>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971116&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>977167</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="n">
+        <v>3</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=977167&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
         <is>
           <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-04-06T02:14:31Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1006389</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1006389&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1009086</t>
+          <t>1100346</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1100346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1019804</t>
+          <t>1129424</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,90 +518,90 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1019804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1129424&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1076391</t>
+          <t>1153930</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1076391&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1153930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1088991</t>
+          <t>1160907</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1088991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1158524</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1158524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1257514</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1257514&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1285611</t>
+          <t>1278649</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1285611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278649&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1367998</t>
+          <t>1285611</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1285611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1421485</t>
+          <t>1334332</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1421485&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1430471</t>
+          <t>1367490</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367490&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1465011</t>
+          <t>1370242</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1465011&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1370242&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1467423</t>
+          <t>1381503</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,33 +708,33 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1467423&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381503&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1471118</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1471118&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1490131</t>
+          <t>1468095</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,52 +746,52 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490131&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1468095&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1490570</t>
+          <t>1485923</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1493821</t>
+          <t>1493061</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1493821&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1493061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1507470</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507470&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1525519</t>
+          <t>1497029</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525519&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1499456</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1499456&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1551224</t>
+          <t>1507477</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1551224&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507477&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1560710</t>
+          <t>1536177</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,33 +879,33 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536177&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1562842</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1567746</t>
+          <t>1574917</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567746&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574917&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1567751</t>
+          <t>1591128</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,52 +936,52 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567751&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591128&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1567752</t>
+          <t>1591199</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567752&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1567784</t>
+          <t>1591388</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1567784&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591388&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1576156</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,14 +993,14 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1587701</t>
+          <t>494868</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1587701&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=494868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1590620</t>
+          <t>510573</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1590620&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>159976</t>
+          <t>610619</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,33 +1050,33 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=610619&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>330009</t>
+          <t>697776</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=330009&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=697776&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>430037</t>
+          <t>761949</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,71 +1088,71 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=430037&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=761949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>769676</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=769676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>771041</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=771041&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>571200</t>
+          <t>819982</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=819982&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>655071</t>
+          <t>830584</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1164,33 +1164,33 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=655071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>701046</t>
+          <t>915286</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=701046&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>729389</t>
+          <t>974715</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1202,14 +1202,14 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=729389&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=974715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>752970</t>
+          <t>999592</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,215 +1221,6 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>786481</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>793949</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="n">
-        <v>2</v>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=793949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>865216</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865216&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>878687</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=878687&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>879692</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>882806</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="n">
-        <v>2</v>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882806&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>910678</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=910678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>919121</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="n">
-        <v>2</v>
-      </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=919121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>937471</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="n">
-        <v>2</v>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>977167</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="n">
-        <v>2</v>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=977167&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="n">
-        <v>2</v>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr">
-        <is>
           <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-04-13T02:29:45Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1009086</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1100346</t>
+          <t>1145623</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,52 +499,52 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1100346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1145623&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1129424</t>
+          <t>1153930</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1129424&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1153930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1153930</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1153930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1160907</t>
+          <t>1285611</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1285611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1413444</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1413444&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1257514</t>
+          <t>1415175</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1257514&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1415175&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1278649</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278649&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1285611</t>
+          <t>1484649</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1285611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1484649&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1334332</t>
+          <t>1497029</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1367490</t>
+          <t>1501202</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1367490&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1501202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1370242</t>
+          <t>1514040</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1370242&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1381503</t>
+          <t>1519380</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381503&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1519380&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1468095</t>
+          <t>1570025</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,52 +746,52 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1468095&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1485923</t>
+          <t>1591199</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1485923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1493061</t>
+          <t>1595237</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1493061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595237&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1595361</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1497029</t>
+          <t>571200</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1499456</t>
+          <t>655071</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1499456&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=655071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1507477</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507477&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1536177</t>
+          <t>848232</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,33 +879,33 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536177&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>859582</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=859582&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1574917</t>
+          <t>915286</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574917&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1591128</t>
+          <t>949125</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,292 +936,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591128&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1591199</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>1591388</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591388&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>469358</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>494868</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=494868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>510573</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>610619</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=610619&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>697776</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=697776&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>761949</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=761949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>769676</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=769676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>771041</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=771041&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>819982</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="n">
-        <v>2</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=819982&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>830584</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="n">
-        <v>2</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830584&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>974715</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=974715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="n">
-        <v>2</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=949125&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-04-20T02:29:53Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1009086</t>
+          <t>1175891</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009086&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1175891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1145623</t>
+          <t>1277901</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,33 +499,33 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1145623&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1277901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1153930</t>
+          <t>1351207</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1153930&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1381378</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1285611</t>
+          <t>1430471</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1285611&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1413444</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1413444&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1415175</t>
+          <t>1478443</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1415175&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1484649</t>
+          <t>1516190</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1484649&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1516190&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1497029</t>
+          <t>1532597</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1501202</t>
+          <t>1539551</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1501202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539551&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1514040</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1519380</t>
+          <t>1591199</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,33 +708,33 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1519380&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>239704</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=239704&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1570025</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1591199</t>
+          <t>300995</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=300995&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1595237</t>
+          <t>463104</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595237&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=463104&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1595361</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,33 +803,33 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>571200</t>
+          <t>707594</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=571200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>655071</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=655071&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>790433</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,33 +860,33 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=790433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>848232</t>
+          <t>915286</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848232&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>859582</t>
+          <t>920115</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,45 +898,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=859582&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>949125</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=949125&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920115&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-04-27T02:33:52Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1175891</t>
+          <t>1031001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1175891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031001&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1277901</t>
+          <t>1047587</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1277901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1351207</t>
+          <t>1244126</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,71 +518,71 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244126&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1381378</t>
+          <t>1312008</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1430471</t>
+          <t>1381151</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1478443</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478443&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1495014</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495014&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1516190</t>
+          <t>1507542</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1516190&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507542&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1532597</t>
+          <t>1508805</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,52 +651,52 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1539551</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539551&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1581394</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1591199</t>
+          <t>802144</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1591199&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=802144&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>239704</t>
+          <t>876141</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=239704&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>941261</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=941261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>300995</t>
+          <t>971121</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,140 +765,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=300995&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>463104</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=463104&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>469358</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>707594</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>764151</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>790433</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=790433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>920115</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920115&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-05-04T02:39:16Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1031001</t>
+          <t>1028222</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031001&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1028222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1047587</t>
+          <t>1074200</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1074200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1244126</t>
+          <t>1160907</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,52 +518,52 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244126&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1312008</t>
+          <t>1198294</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1381151</t>
+          <t>1294347</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1294347&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1355692</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1355692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1372929</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1495014</t>
+          <t>1375255</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495014&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1507542</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1507542&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1508805</t>
+          <t>1454208</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,71 +651,71 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1454208&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1468095</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1468095&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1581394</t>
+          <t>1495296</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495296&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>802144</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=802144&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>1565061</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1565061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>941261</t>
+          <t>1576901</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=941261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>971121</t>
+          <t>1581394</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,7 +765,121 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>352570</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>486442</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=486442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>764151</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>943950</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=943950&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-05-11T02:53:27Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1028222</t>
+          <t>1209526</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1028222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1074200</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1074200&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1160907</t>
+          <t>1262277</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1160907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1262277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1198294</t>
+          <t>1278602</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1198294&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1294347</t>
+          <t>1312061</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1294347&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1355692</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,7 +575,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1355692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -601,26 +601,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1375255</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1508805</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1454208</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1454208&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1468095</t>
+          <t>1553965</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1468095&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553965&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1495296</t>
+          <t>1570025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495296&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1576901</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1565061</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1565061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1576901</t>
+          <t>40910</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=40910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1581394</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>352570</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>830594</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,33 +803,33 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>486442</t>
+          <t>975065</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=486442&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975065&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>990242</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,45 +841,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>943950</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=943950&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=990242&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-05-18T03:00:30Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1209526</t>
+          <t>1019804</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1019804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1026153</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1026153&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1262277</t>
+          <t>1263891</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1262277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1263891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1278602</t>
+          <t>1351207</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1312061</t>
+          <t>1361978</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312061&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1423164</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1423164&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1372929</t>
+          <t>1486307</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1486791</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1508805</t>
+          <t>1490581</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1498127</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498127&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1553965</t>
+          <t>1536177</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553965&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536177&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1570025</t>
+          <t>412675</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=412675&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1576901</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1576901&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>40910</t>
+          <t>689351</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,33 +746,33 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=40910&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=689351&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>804994</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>824679</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,64 +784,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>830594</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=830594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>975065</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975065&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>990242</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=990242&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-05-25T03:34:26Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1019804</t>
+          <t>1020352</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1019804&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1020352&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1026153</t>
+          <t>1184431</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1026153&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1263891</t>
+          <t>1209526</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1263891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1351207</t>
+          <t>1244132</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244132&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1361978</t>
+          <t>1271614</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1271614&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1423164</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1423164&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1486307</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486307&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1486791</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1490581</t>
+          <t>1476637</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476637&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1498127</t>
+          <t>1483337</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498127&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1536177</t>
+          <t>1484916</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1536177&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1484916&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>412675</t>
+          <t>1575412</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,7 +689,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=412675&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
@@ -715,7 +715,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>689351</t>
+          <t>849891</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,33 +746,33 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=689351&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=849891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>804994</t>
+          <t>865097</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>824679</t>
+          <t>879605</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,7 +784,45 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879605&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>881907</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>920049</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920049&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-06-01T03:45:50Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +487,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1184431</t>
+          <t>1031529</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031529&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1209526</t>
+          <t>1127852</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1127852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1244132</t>
+          <t>1206680</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244132&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1206680&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1271614</t>
+          <t>1209526</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1271614&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1286676</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,52 +594,52 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1299630</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1299630&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1476637</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476637&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1483337</t>
+          <t>1312008</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1483337&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1484916</t>
+          <t>1344943</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1484916&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1575412</t>
+          <t>1372828</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1381412</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>1417234</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1417234&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>849891</t>
+          <t>1497029</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=849891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>865097</t>
+          <t>1501319</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=865097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1501319&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>879605</t>
+          <t>1513080</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879605&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1513080&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>881907</t>
+          <t>455575</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,26 +803,178 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=881907&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=455575&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>920049</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920049&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>712697</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=712697&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>804994</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>824644</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>878687</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=878687&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>879581</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>895147</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>918250</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=918250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-06-08T03:42:47Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1020352</t>
+          <t>1083730</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1020352&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1083730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1031529</t>
+          <t>1255179</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031529&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1255179&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1127852</t>
+          <t>1290822</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,33 +518,33 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1127852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290822&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1206680</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1206680&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1209526</t>
+          <t>1334530</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334530&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1394289</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394289&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1286676</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1299630</t>
+          <t>242415</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,33 +613,33 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1299630&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1312008</t>
+          <t>352545</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1344943</t>
+          <t>716574</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=716574&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1372828</t>
+          <t>761949</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,292 +689,64 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=761949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1381412</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381412&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1417234</t>
+          <t>824644</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1417234&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1497029</t>
+          <t>882800</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497029&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1501319</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1501319&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1513080</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1513080&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>455575</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=455575&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>469358</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>712697</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=712697&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>804994</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>824644</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>878687</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=878687&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>879581</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879581&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>895147</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=895147&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>918250</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=918250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882800&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-06-15T03:59:31Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1083730</t>
+          <t>1009430</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1083730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009430&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1255179</t>
+          <t>1076391</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1255179&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1076391&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1290822</t>
+          <t>1146718</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,52 +518,52 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290822&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1146718&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1297231</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1297231&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1334530</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334530&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1394289</t>
+          <t>1404331</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394289&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404331&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1404947</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404947&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>242415</t>
+          <t>1435726</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,33 +613,33 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>352545</t>
+          <t>1498884</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498884&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>716574</t>
+          <t>1514460</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=716574&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514460&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>761949</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,52 +689,52 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=761949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>1575671</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575671&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>824644</t>
+          <t>1595747</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>882800</t>
+          <t>352545</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,7 +746,159 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882800&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>358474</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=358474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>493192</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=493192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>621809</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>860698</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>975970</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-06-22T03:57:51Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1009430</t>
+          <t>1019263</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1009430&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1019263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1076391</t>
+          <t>1091204</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,33 +499,33 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1076391&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1091204&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1146718</t>
+          <t>1361978</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1146718&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1297231</t>
+          <t>1387361</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1297231&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1387361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1393661</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1393661&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1404331</t>
+          <t>1400298</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404331&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1400298&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1404947</t>
+          <t>1426319</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,52 +594,52 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1404947&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1426319&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1435726</t>
+          <t>1430471</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1466482</t>
+          <t>1490578</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490578&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1498884</t>
+          <t>1494342</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498884&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1514460</t>
+          <t>1514040</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514460&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1581274</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581274&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1575671</t>
+          <t>1588421</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1575671&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1588421&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1595747</t>
+          <t>1589504</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1595747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>352545</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>358474</t>
+          <t>720178</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=358474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=720178&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>752970</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>493192</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=493192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>816750</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,26 +841,26 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=816750&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>860698</t>
+          <t>824644</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860698&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>975970</t>
+          <t>976980</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,7 +898,26 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-06-29T03:40:19Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1019263</t>
+          <t>1109881</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,52 +480,52 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1019263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1109881&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1091204</t>
+          <t>1150628</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1091204&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1361978</t>
+          <t>1152259</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361978&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1387361</t>
+          <t>1170299</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1387361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170299&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1393661</t>
+          <t>1176790</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1393661&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176790&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1400298</t>
+          <t>1232243</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1400298&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1426319</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1426319&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1430471</t>
+          <t>1345526</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,52 +613,52 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1430471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1490578</t>
+          <t>1375251</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490578&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375251&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1494342</t>
+          <t>1375256</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1494342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375256&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1514040</t>
+          <t>1394366</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394366&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1581274</t>
+          <t>1396441</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1581274&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1396441&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1588421</t>
+          <t>1397305</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1588421&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1397305&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1589504</t>
+          <t>1402376</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1402376&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>1478310</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478310&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>720178</t>
+          <t>1478506</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=720178&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478506&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>752970</t>
+          <t>1490578</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490578&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>1504322</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,33 +803,33 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1504322&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>1508481</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>816750</t>
+          <t>1511772</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=816750&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1511772&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>824644</t>
+          <t>1514040</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,33 +860,33 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824644&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>1514460</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514460&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>976980</t>
+          <t>1525485</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525485&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>999592</t>
+          <t>1526923</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,7 +917,425 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1544832</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1560710</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1580751</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580751&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1586318</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586318&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1606886</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1610285</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1610285&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>340813</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=340813&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>352545</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>621809</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>707031</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707031&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>720787</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=720787&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>779081</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=779081&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>804994</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>815202</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=815202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>837561</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=837561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>870084</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=870084&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>875594</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=875594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>882800</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882800&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>902672</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=902672&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>910678</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=910678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>952369</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=952369&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-07-06T02:55:44Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1109881</t>
+          <t>1031001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,52 +480,52 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1109881&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031001&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1150628</t>
+          <t>1152259</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1152259</t>
+          <t>1232243</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1170299</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170299&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1176790</t>
+          <t>1290730</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1176790&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1298088</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1298088&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1307555</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,71 +594,71 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1345526</t>
+          <t>1312008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1375251</t>
+          <t>1351207</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375251&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1375256</t>
+          <t>1471014</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1375256&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1471014&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1394366</t>
+          <t>1471679</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1394366&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1471679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1396441</t>
+          <t>1482438</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1396441&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1482438&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1397305</t>
+          <t>1486791</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1397305&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1402376</t>
+          <t>1498332</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1402376&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1478310</t>
+          <t>1570728</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478310&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570728&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1478506</t>
+          <t>1573923</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478506&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1573923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1490578</t>
+          <t>1604241</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1490578&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1604241&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1504322</t>
+          <t>242415</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1504322&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1508481</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1511772</t>
+          <t>575007</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1511772&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=575007&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1514040</t>
+          <t>669005</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,33 +860,33 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=669005&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1514460</t>
+          <t>824679</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514460&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1525485</t>
+          <t>879692</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1525485&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1526923</t>
+          <t>975970</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,425 +917,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>1544832</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1560710</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>1580751</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580751&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>1586318</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586318&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>1606886</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>1610285</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1610285&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>340813</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=340813&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>352545</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>621809</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>707031</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707031&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>720787</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=720787&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>779081</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="n">
-        <v>2</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=779081&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>804994</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="n">
-        <v>3</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>815202</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=815202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>837561</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=837561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>870084</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="n">
-        <v>2</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=870084&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>875594</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=875594&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>876141</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="n">
-        <v>2</v>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>882800</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=882800&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>902672</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=902672&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>910678</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=910678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>952369</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="n">
-        <v>2</v>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=952369&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-07-13T02:31:59Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1031001</t>
+          <t>1037522</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1031001&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1037522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1152259</t>
+          <t>1040773</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1040773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1232243</t>
+          <t>1209526</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1232243&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1213353</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213353&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1290730</t>
+          <t>1255535</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1290730&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1255535&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1298088</t>
+          <t>1309827</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1298088&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1309827&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1307555</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1312008</t>
+          <t>1389833</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1312008&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389833&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1351207</t>
+          <t>1436341</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1436341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1471014</t>
+          <t>1500483</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1471014&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1471679</t>
+          <t>1529093</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1471679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1482438</t>
+          <t>1535799</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1482438&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1535799&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1486791</t>
+          <t>1546562</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486791&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546562&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1498332</t>
+          <t>1589504</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,71 +727,71 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1570728</t>
+          <t>1603180</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1570728&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1573923</t>
+          <t>1603192</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1573923&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1604241</t>
+          <t>242415</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1604241&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>242415</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>708509</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=708509&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>575007</t>
+          <t>713850</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=575007&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=713850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>669005</t>
+          <t>824679</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=669005&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>824679</t>
+          <t>826992</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826992&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>879692</t>
+          <t>848767</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=879692&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848767&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>975970</t>
+          <t>968713</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,7 +917,26 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=975970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=968713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>971145</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971145&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-07-20T03:39:53Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1037522</t>
+          <t>1023776</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1037522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1023776&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1040773</t>
+          <t>1037522</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1040773&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1037522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1209526</t>
+          <t>1272972</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1209526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1272972&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1213353</t>
+          <t>1486376</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,52 +537,52 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1213353&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486376&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1255535</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1255535&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1309827</t>
+          <t>1500483</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1309827&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1514040</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1389833</t>
+          <t>1529093</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389833&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1436341</t>
+          <t>1574267</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1436341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574267&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1500483</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,33 +651,33 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1529093</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1535799</t>
+          <t>722492</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1535799&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722492&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1546562</t>
+          <t>804994</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546562&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1589504</t>
+          <t>815586</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,216 +727,45 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=815586&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1603180</t>
+          <t>837561</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=837561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1603192</t>
+          <t>976980</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>242415</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>4</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=242415&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>621809</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>708509</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=708509&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>713850</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=713850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>824679</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>826992</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=826992&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>848767</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=848767&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>968713</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=968713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>971145</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971145&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-07-27T02:40:51Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1023776</t>
+          <t>1047034</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1023776&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1037522</t>
+          <t>1047473</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1037522&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047473&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1272972</t>
+          <t>1057279</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1272972&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1057279&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1486376</t>
+          <t>1090474</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486376&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1090474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1107283</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1500483</t>
+          <t>1179458</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1514040</t>
+          <t>1246450</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,33 +594,33 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1514040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1246450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1529093</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1574267</t>
+          <t>1278602</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574267&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>1286676</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,33 +651,33 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>1329122</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>722492</t>
+          <t>1352197</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,33 +689,33 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722492&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1352197&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>804994</t>
+          <t>1378864</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804994&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1378864&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>815586</t>
+          <t>1387361</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=815586&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1387361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>837561</t>
+          <t>1429486</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=837561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1429486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>976980</t>
+          <t>1478705</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,7 +765,444 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478705&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1486025</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1486152</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486152&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1488550</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488550&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1491899</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1508229</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508229&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1526108</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1529093</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1544832</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1554418</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1554418&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1602612</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1603180</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>599450</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=599450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>621809</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>707031</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>4</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707031&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>876141</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>908952</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908952&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>909900</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=909900&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>984333</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=984333&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>991747</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-08-03T02:34:17Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1047034</t>
+          <t>1047473</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047473&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1047473</t>
+          <t>1084121</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047473&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1057279</t>
+          <t>1102108</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1057279&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1102108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1090474</t>
+          <t>1107283</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1090474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1107283</t>
+          <t>1133161</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1133161&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1179458</t>
+          <t>1152259</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1179458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1246450</t>
+          <t>1162292</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,52 +594,52 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1246450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1244132</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244132&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1278602</t>
+          <t>1307555</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1278602&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1286676</t>
+          <t>1329122</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1329122</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1352197</t>
+          <t>1354859</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1352197&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1378864</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1378864&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1387361</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,33 +727,33 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1387361&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1429486</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1429486&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1478705</t>
+          <t>1478462</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,52 +765,52 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478705&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1486025</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486025&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1486152</t>
+          <t>1529093</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486152&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1488550</t>
+          <t>1541431</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,33 +822,33 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488550&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1563342</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1563342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1508229</t>
+          <t>1574068</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,52 +860,52 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508229&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1526108</t>
+          <t>1579332</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1579332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1529093</t>
+          <t>1586128</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586128&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1599875</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1599875&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1554418</t>
+          <t>1602612</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1554418&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1602612</t>
+          <t>1606936</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,33 +955,33 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606936&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1603180</t>
+          <t>584975</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=584975&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>684433</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,14 +993,14 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>722492</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,33 +1012,33 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722492&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>599450</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=599450&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>791604</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,33 +1050,33 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=791604&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>707031</t>
+          <t>799309</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=707031&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=799309&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>876141</t>
+          <t>811161</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=876141&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=811161&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>908952</t>
+          <t>821096</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908952&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=821096&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>909900</t>
+          <t>849891</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,33 +1126,33 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=909900&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=849891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>937471</t>
+          <t>915286</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>984333</t>
+          <t>944166</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1164,45 +1164,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=984333&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>991747</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>999592</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944166&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-08-10T01:28:07Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1047473</t>
+          <t>1049381</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047473&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1084121</t>
+          <t>1150628</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1084121&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1102108</t>
+          <t>1152967</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1102108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152967&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1107283</t>
+          <t>1172375</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1107283&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1172375&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1133161</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1133161&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1152259</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152259&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1162292</t>
+          <t>1342142</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1162292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1342142&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1244132</t>
+          <t>1345526</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,33 +613,33 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244132&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1307555</t>
+          <t>1347117</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307555&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1329122</t>
+          <t>1475939</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,52 +651,52 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1475939&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1354859</t>
+          <t>1497579</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1354859&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497579&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1534946</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1534946&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1547570</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,90 +727,90 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1466482</t>
+          <t>1554394</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1554394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1478462</t>
+          <t>1586216</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478462&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586216&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1529093</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1541431</t>
+          <t>543781</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=543781&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1563342</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,33 +841,33 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1563342&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1574068</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1579332</t>
+          <t>793949</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1579332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=793949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1586128</t>
+          <t>819982</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586128&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=819982&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1599875</t>
+          <t>880642</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,14 +917,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1599875&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1602612</t>
+          <t>934091</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=934091&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1606936</t>
+          <t>947561</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,216 +955,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606936&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>584975</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=584975&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>684433</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>722492</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=722492&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>764151</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>5</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>791604</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=791604&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>799309</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=799309&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>811161</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=811161&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>821096</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=821096&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>849891</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=849891&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="n">
-        <v>4</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>944166</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="n">
-        <v>2</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944166&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=947561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-08-17T01:06:53Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1049381</t>
+          <t>100458</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1150628</t>
+          <t>1029937</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1150628&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029937&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1152967</t>
+          <t>1049381</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1152967&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1172375</t>
+          <t>1093803</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1172375&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1170247</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1275466</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1275466&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1342142</t>
+          <t>1276718</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1342142&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1276718&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1345526</t>
+          <t>1342142</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1345526&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1342142&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1347117</t>
+          <t>1465349</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,71 +632,71 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347117&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1465349&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1475939</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1475939&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1495517</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495517&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1497579</t>
+          <t>1503123</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497579&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1503123&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1534946</t>
+          <t>1539679</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1534946&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1547570</t>
+          <t>1556887</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,52 +727,52 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547570&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1556887&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1554394</t>
+          <t>1578263</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1554394&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1586216</t>
+          <t>1580286</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586216&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1586216</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586216&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>1589504</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,33 +803,33 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>543781</t>
+          <t>1602612</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=543781&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>1603180</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,33 +841,33 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>1607268</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1607268&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>793949</t>
+          <t>1612256</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=793949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1612256&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>819982</t>
+          <t>239704</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,52 +898,52 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=819982&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=239704&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>880642</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=880642&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>934091</t>
+          <t>322983</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=934091&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=322983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>947561</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,7 +955,178 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=947561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>764151</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>786481</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>857942</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>913113</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=913113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>915034</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>956535</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=956535&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>968713</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=968713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>976980</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-08-24T01:06:53Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100458</t>
+          <t>1029103</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029103&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1029937</t>
+          <t>1181236</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,52 +499,52 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029937&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1049381</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1093803</t>
+          <t>1329122</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1093803&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1170247</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,33 +556,33 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1275466</t>
+          <t>1502050</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1275466&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502050&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1276718</t>
+          <t>1512422</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1276718&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1512422&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1342142</t>
+          <t>1562850</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1342142&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1465349</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1465349&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1495517</t>
+          <t>586189</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1495517&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=586189&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1503123</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1503123&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1539679</t>
+          <t>633093</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=633093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1556887</t>
+          <t>650672</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1556887&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=650672&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1578263</t>
+          <t>768387</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768387&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1580286</t>
+          <t>822138</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,368 +765,26 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=822138&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1586216</t>
+          <t>915286</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586216&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1589504</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1602612</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1603180</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1607268</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1607268&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>1612256</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1612256&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>239704</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=239704&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>255970</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>322983</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=322983&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>469358</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>545355</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>764151</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>786481</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>857942</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857942&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>913113</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=913113&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>915034</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>956535</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=956535&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>968713</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=968713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>976980</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=976980&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-08-31T03:27:35Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1029103</t>
+          <t>1008277</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1029103&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1008277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1181236</t>
+          <t>1142809</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,52 +499,52 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1181236&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1142809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1281098</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1281098&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1329122</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1329122&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1341083</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341083&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1502050</t>
+          <t>1420726</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1502050&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1420726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1512422</t>
+          <t>1436341</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1512422&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1436341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1562850</t>
+          <t>1458521</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1562850&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1458521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1478705</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478705&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>1624715</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1624715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>586189</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=586189&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>633093</t>
+          <t>550715</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=633093&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=550715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>650672</t>
+          <t>868202</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=650672&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=868202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>768387</t>
+          <t>920040</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=768387&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>822138</t>
+          <t>999592</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,26 +765,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=822138&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>915286</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>